<commit_message>
Update daily Zee Business signals
</commit_message>
<xml_diff>
--- a/zeebiz_live_stocks.xlsx
+++ b/zeebiz_live_stocks.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Latest by Stock" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Website Signals'!$A$1:$J$938</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Website Signals'!$A$1:$J$1002</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Latest by Stock'!$A$1:$J$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J938"/>
+  <dimension ref="A1:J1002"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -33999,7 +33999,6 @@
       <c r="F783" t="n">
         <v>360</v>
       </c>
-      <c r="G783" t="inlineStr"/>
       <c r="H783" t="inlineStr">
         <is>
           <t>Indian Hume Pipe 387.65 15.50 BUY TGT 405 SL 360</t>
@@ -34041,7 +34040,6 @@
       <c r="F784" t="n">
         <v>335</v>
       </c>
-      <c r="G784" t="inlineStr"/>
       <c r="H784" t="inlineStr">
         <is>
           <t>Sunflag Iron 346.55 6.90 BUY TGT 370 SL 335</t>
@@ -34083,7 +34081,6 @@
       <c r="F785" t="n">
         <v>480</v>
       </c>
-      <c r="G785" t="inlineStr"/>
       <c r="H785" t="inlineStr">
         <is>
           <t>Super KOOL MEHUL Hind Copper 520.25 1.22% BUY TGT 600 SL 480</t>
@@ -34125,7 +34122,6 @@
       <c r="F786" t="n">
         <v>2005</v>
       </c>
-      <c r="G786" t="inlineStr"/>
       <c r="H786" t="inlineStr">
         <is>
           <t>BEML 2033.30 BUY TGT 2078 SL 2005</t>
@@ -34167,7 +34163,6 @@
       <c r="F787" t="n">
         <v>2005</v>
       </c>
-      <c r="G787" t="inlineStr"/>
       <c r="H787" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर BEML 2032.20 62.00 BUY TGT 2070 SL 2005</t>
@@ -34209,7 +34204,6 @@
       <c r="F788" t="n">
         <v>262</v>
       </c>
-      <c r="G788" t="inlineStr"/>
       <c r="H788" t="inlineStr">
         <is>
           <t>ITC Fut 267.90 0.80 BUY TGT 277 SL 262</t>
@@ -34242,11 +34236,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D789" t="inlineStr"/>
       <c r="E789" t="n">
         <v>158.5</v>
       </c>
-      <c r="G789" t="inlineStr"/>
       <c r="H789" t="inlineStr">
         <is>
           <t>जैन साब के GEMS
@@ -34283,11 +34275,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D790" t="inlineStr"/>
       <c r="E790" t="n">
         <v>930</v>
       </c>
-      <c r="G790" t="inlineStr"/>
       <c r="H790" t="inlineStr">
         <is>
           <t>जैन साब के GEMS
@@ -34334,7 +34324,6 @@
       <c r="F791" t="n">
         <v>20200</v>
       </c>
-      <c r="G791" t="inlineStr"/>
       <c r="H791" t="inlineStr">
         <is>
           <t>जय का JACKPOT
@@ -34381,7 +34370,6 @@
       <c r="F792" t="n">
         <v>20200</v>
       </c>
-      <c r="G792" t="inlineStr"/>
       <c r="H792" t="inlineStr">
         <is>
           <t>जय का JACKPOT
@@ -34428,7 +34416,6 @@
       <c r="F793" t="n">
         <v>20200</v>
       </c>
-      <c r="G793" t="inlineStr"/>
       <c r="H793" t="inlineStr">
         <is>
           <t>जय का JACKPOT
@@ -34577,7 +34564,6 @@
       <c r="F796" t="n">
         <v>425</v>
       </c>
-      <c r="G796" t="inlineStr"/>
       <c r="H796" t="inlineStr">
         <is>
           <t>Super Kool Mehul
@@ -34624,7 +34610,6 @@
       <c r="F797" t="n">
         <v>425</v>
       </c>
-      <c r="G797" t="inlineStr"/>
       <c r="H797" t="inlineStr">
         <is>
           <t>Super Kool Mehul
@@ -34671,7 +34656,6 @@
       <c r="F798" t="n">
         <v>425</v>
       </c>
-      <c r="G798" t="inlineStr"/>
       <c r="H798" t="inlineStr">
         <is>
           <t>मेहुल कोटारी की राय
@@ -34718,7 +34702,6 @@
       <c r="F799" t="n">
         <v>425</v>
       </c>
-      <c r="G799" t="inlineStr"/>
       <c r="H799" t="inlineStr">
         <is>
           <t>मेहुल कोटारी की राय
@@ -34765,7 +34748,6 @@
       <c r="F800" t="n">
         <v>335</v>
       </c>
-      <c r="G800" t="inlineStr"/>
       <c r="H800" t="inlineStr">
         <is>
           <t>सदाबहार सेठी सा'ब
@@ -34904,7 +34886,6 @@
       <c r="F803" t="n">
         <v>360</v>
       </c>
-      <c r="G803" t="inlineStr"/>
       <c r="H803" t="inlineStr">
         <is>
           <t>सदाबहार सेठी साब Indian Hume Pipe 386.05 13.90 BUY TGT 405 SL 360</t>
@@ -35038,7 +35019,6 @@
       <c r="F806" t="n">
         <v>480</v>
       </c>
-      <c r="G806" t="inlineStr"/>
       <c r="H806" t="inlineStr">
         <is>
           <t>Super KOOL MEHUL
@@ -35088,7 +35068,6 @@
       <c r="F807" t="n">
         <v>480</v>
       </c>
-      <c r="G807" t="inlineStr"/>
       <c r="H807" t="inlineStr">
         <is>
           <t>Super Kool Mehul
@@ -35135,7 +35114,6 @@
       <c r="F808" t="n">
         <v>351</v>
       </c>
-      <c r="G808" t="inlineStr"/>
       <c r="H808" t="inlineStr">
         <is>
           <t>सच्चितानंद उस्तेकर की राय Federal Bank Fut खरीदें PRICE 355.75 TARGET 362/370 STOP LOSS 351</t>
@@ -35177,7 +35155,6 @@
       <c r="F809" t="n">
         <v>351</v>
       </c>
-      <c r="G809" t="inlineStr"/>
       <c r="H809" t="inlineStr">
         <is>
           <t>सच्चितानंद उस्तेकर की राय Federal Bank Fut खरीदें PRICE 355.75 TARGET 362/370 STOP LOSS 351</t>
@@ -35403,7 +35380,6 @@
       <c r="F814" t="n">
         <v>212</v>
       </c>
-      <c r="G814" t="inlineStr"/>
       <c r="H814" t="inlineStr">
         <is>
           <t>TRADING CALL Piramal Pharma खरीदें PRICE 217.30 TARGET 222/225 STOP LOSS 212</t>
@@ -35445,7 +35421,6 @@
       <c r="F815" t="n">
         <v>212</v>
       </c>
-      <c r="G815" t="inlineStr"/>
       <c r="H815" t="inlineStr">
         <is>
           <t>TRADING CALL Piramal Pharma खरीदें PRICE 217.30 TARGET 222/225 STOP LOSS 212</t>
@@ -35487,7 +35462,6 @@
       <c r="F816" t="n">
         <v>710</v>
       </c>
-      <c r="G816" t="inlineStr"/>
       <c r="H816" t="inlineStr">
         <is>
           <t>शिवांगी सारदा की पसंद Indian Hotels खरीदें PRICE 724.40 TARGET 750 STOP LOSS 710</t>
@@ -35529,7 +35503,6 @@
       <c r="F817" t="n">
         <v>4920</v>
       </c>
-      <c r="G817" t="inlineStr"/>
       <c r="H817" t="inlineStr">
         <is>
           <t>शिवांगी सारदा की पसंद Titan खरीदें PRICE 5025.00 TARGET 5250 STOP LOSS 4920</t>
@@ -35571,7 +35544,6 @@
       <c r="F818" t="n">
         <v>320</v>
       </c>
-      <c r="G818" t="inlineStr"/>
       <c r="H818" t="inlineStr">
         <is>
           <t>शिवांगी सारदा की राय
@@ -35618,7 +35590,6 @@
       <c r="F819" t="n">
         <v>1000</v>
       </c>
-      <c r="G819" t="inlineStr"/>
       <c r="H819" t="inlineStr">
         <is>
           <t>शिवांगी सारदा की राय SBI 1020.60 ▼ 1.35% HOLD TARGET 1060 STOP LOSS 1000</t>
@@ -35660,7 +35631,6 @@
       <c r="F820" t="n">
         <v>1111</v>
       </c>
-      <c r="G820" t="inlineStr"/>
       <c r="H820" t="inlineStr">
         <is>
           <t>शिवांगी सारदा की राय
@@ -35707,7 +35677,6 @@
       <c r="F821" t="n">
         <v>1800</v>
       </c>
-      <c r="G821" t="inlineStr"/>
       <c r="H821" t="inlineStr">
         <is>
           <t>अक्षय भागवत की राय
@@ -35754,7 +35723,6 @@
       <c r="F822" t="n">
         <v>1800</v>
       </c>
-      <c r="G822" t="inlineStr"/>
       <c r="H822" t="inlineStr">
         <is>
           <t>अक्षय भागवत की राय
@@ -35801,7 +35769,6 @@
       <c r="F823" t="n">
         <v>55</v>
       </c>
-      <c r="G823" t="inlineStr"/>
       <c r="H823" t="inlineStr">
         <is>
           <t>छोटा ऑप्शन बड़ी कमाई
@@ -35847,7 +35814,6 @@
       <c r="F824" t="n">
         <v>55</v>
       </c>
-      <c r="G824" t="inlineStr"/>
       <c r="H824" t="inlineStr">
         <is>
           <t>छोटा ऑप्शन बड़ी कमाई
@@ -35893,7 +35859,6 @@
       <c r="F825" t="n">
         <v>203</v>
       </c>
-      <c r="G825" t="inlineStr"/>
       <c r="H825" t="inlineStr">
         <is>
           <t>ITC Fut PRICE 268.3 TARGET 277/203</t>
@@ -35935,7 +35900,6 @@
       <c r="F826" t="n">
         <v>520</v>
       </c>
-      <c r="G826" t="inlineStr"/>
       <c r="H826" t="inlineStr">
         <is>
           <t>GNA Axles @ 536 खरीदें STOP LOSS 520 TARGET 560 DURATION -- GNA Axles 540.50 8.05</t>
@@ -35977,7 +35941,6 @@
       <c r="F827" t="n">
         <v>1000</v>
       </c>
-      <c r="G827" t="inlineStr"/>
       <c r="H827" t="inlineStr">
         <is>
           <t>Mangalam Cem खरीदें PRICE 1109.40 TARGET 1200/1250 STOP LOSS 1000 नवनीत मुनोत MD &amp; CEO HDFC AMC COMING UP</t>
@@ -36019,7 +35982,6 @@
       <c r="F828" t="n">
         <v>1000</v>
       </c>
-      <c r="G828" t="inlineStr"/>
       <c r="H828" t="inlineStr">
         <is>
           <t>10 की कमाई Mangalam Cem खरीदें PRICE 1110.00 TARGET 1200/1250 STOP LOSS 1000</t>
@@ -36061,7 +36023,6 @@
       <c r="F829" t="n">
         <v>422</v>
       </c>
-      <c r="G829" t="inlineStr"/>
       <c r="H829" t="inlineStr">
         <is>
           <t>विशेष के विशेष
@@ -36108,7 +36069,6 @@
       <c r="F830" t="n">
         <v>422</v>
       </c>
-      <c r="G830" t="inlineStr"/>
       <c r="H830" t="inlineStr">
         <is>
           <t>विशेष के विशेष
@@ -36152,7 +36112,6 @@
       <c r="E831" t="n">
         <v>930</v>
       </c>
-      <c r="G831" t="inlineStr"/>
       <c r="H831" t="inlineStr">
         <is>
           <t>जैन साब के GEMS
@@ -36196,7 +36155,6 @@
       <c r="E832" t="n">
         <v>930</v>
       </c>
-      <c r="G832" t="inlineStr"/>
       <c r="H832" t="inlineStr">
         <is>
           <t>जैन साब के GEMS
@@ -36243,7 +36201,6 @@
       <c r="F833" t="n">
         <v>1840</v>
       </c>
-      <c r="G833" t="inlineStr"/>
       <c r="H833" t="inlineStr">
         <is>
           <t>जय का JACKPOT Oberoi Realty Fut 1854.30 31.30 BUY TGT 1930 SL 1840</t>
@@ -36285,7 +36242,6 @@
       <c r="F834" t="n">
         <v>1960</v>
       </c>
-      <c r="G834" t="inlineStr"/>
       <c r="H834" t="inlineStr">
         <is>
           <t>1 की कमाई
@@ -36332,7 +36288,6 @@
       <c r="F835" t="n">
         <v>1960</v>
       </c>
-      <c r="G835" t="inlineStr"/>
       <c r="H835" t="inlineStr">
         <is>
           <t>10 की कमाई Alkyl Amines खरीदें PRICE 2028.40 TARGET 2100/2150 STOP LOSS 1960 MARKET MENTORS नवनीत मुनोत MD &amp; CEO HDFC AMC 11 AM</t>
@@ -36374,7 +36329,6 @@
       <c r="F836" t="n">
         <v>500</v>
       </c>
-      <c r="G836" t="inlineStr"/>
       <c r="H836" t="inlineStr">
         <is>
           <t>LONG MIDCAP STOCKS
@@ -36416,7 +36370,6 @@
       <c r="D837" t="n">
         <v>603.5</v>
       </c>
-      <c r="G837" t="inlineStr"/>
       <c r="H837" t="inlineStr">
         <is>
           <t>Innogene खरीदें STOP LOSS 500 TARGET ₹50</t>
@@ -36449,14 +36402,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D838" t="inlineStr"/>
       <c r="E838" t="n">
         <v>340</v>
       </c>
       <c r="F838" t="n">
         <v>270</v>
       </c>
-      <c r="G838" t="inlineStr"/>
       <c r="H838" t="inlineStr">
         <is>
           <t>POSITIONAL MIDCAP STOCK SCI खरीदें STOP LOSS 270 TARGET 340 DURATION</t>
@@ -36498,7 +36449,6 @@
       <c r="F839" t="n">
         <v>380</v>
       </c>
-      <c r="G839" t="inlineStr"/>
       <c r="H839" t="inlineStr">
         <is>
           <t>LONG MIDCAP STOCKS
@@ -36535,7 +36485,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D840" t="inlineStr"/>
       <c r="E840" t="n">
         <v>240</v>
       </c>
@@ -36579,7 +36528,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D841" t="inlineStr"/>
       <c r="E841" t="n">
         <v>270</v>
       </c>
@@ -36632,7 +36580,6 @@
       <c r="F842" t="n">
         <v>500</v>
       </c>
-      <c r="G842" t="inlineStr"/>
       <c r="H842" t="inlineStr">
         <is>
           <t>सौमिल मेहता की राय Indegene खरीदें STOP LOSS 500 TARGET 850 DURATION -- Indegene 606.25 0.14%</t>
@@ -36665,14 +36612,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D843" t="inlineStr"/>
       <c r="E843" t="n">
         <v>550</v>
       </c>
       <c r="F843" t="n">
         <v>380</v>
       </c>
-      <c r="G843" t="inlineStr"/>
       <c r="H843" t="inlineStr">
         <is>
           <t>LONG MIDCAP STOCKS
@@ -36709,7 +36654,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D844" t="inlineStr"/>
       <c r="E844" t="n">
         <v>550</v>
       </c>
@@ -36766,7 +36710,6 @@
       <c r="F845" t="n">
         <v>422</v>
       </c>
-      <c r="G845" t="inlineStr"/>
       <c r="H845" t="inlineStr">
         <is>
           <t>Kotak Bank Fut 425.25 1.50 BUY TGT 432 SL 422</t>
@@ -36808,7 +36751,6 @@
       <c r="F846" t="n">
         <v>606</v>
       </c>
-      <c r="G846" t="inlineStr"/>
       <c r="H846" t="inlineStr">
         <is>
           <t>10 की कमाई UFLEX @ 656-660 खरीदें STOP LOSS 606 TARGET 720/750 Uflex 667.25 ▲ 3.36%</t>
@@ -36847,7 +36789,6 @@
       <c r="E847" t="n">
         <v>400</v>
       </c>
-      <c r="G847" t="inlineStr"/>
       <c r="H847" t="inlineStr">
         <is>
           <t>Eternal TARGET 400 ALLOCATION 25%</t>
@@ -36886,7 +36827,6 @@
       <c r="E848" t="n">
         <v>1500</v>
       </c>
-      <c r="G848" t="inlineStr"/>
       <c r="H848" t="inlineStr">
         <is>
           <t>SID की SIP MapmyIndia CMP 985.20 TARGET 1500 25% ALLOCATION</t>
@@ -36925,7 +36865,6 @@
       <c r="E849" t="n">
         <v>2000</v>
       </c>
-      <c r="G849" t="inlineStr"/>
       <c r="H849" t="inlineStr">
         <is>
           <t>SID की SIP, Affle 3i, CMP 1534.00, TARGET 2000, 25% ALLOCATION</t>
@@ -36964,7 +36903,6 @@
       <c r="E850" t="n">
         <v>2000</v>
       </c>
-      <c r="G850" t="inlineStr"/>
       <c r="H850" t="inlineStr">
         <is>
           <t>SID की SIP
@@ -37007,7 +36945,6 @@
       <c r="E851" t="n">
         <v>230</v>
       </c>
-      <c r="G851" t="inlineStr"/>
       <c r="H851" t="inlineStr">
         <is>
           <t>SID की SIP Meesho CMP 206.54 TARGET 230 25% ALLOCATION</t>
@@ -37046,7 +36983,6 @@
       <c r="E852" t="n">
         <v>400</v>
       </c>
-      <c r="G852" t="inlineStr"/>
       <c r="H852" t="inlineStr">
         <is>
           <t>SID को SIP
@@ -37090,7 +37026,6 @@
       <c r="E853" t="n">
         <v>930</v>
       </c>
-      <c r="G853" t="inlineStr"/>
       <c r="H853" t="inlineStr">
         <is>
           <t>जैन साब के GEMS
@@ -37137,7 +37072,6 @@
       <c r="F854" t="n">
         <v>1840</v>
       </c>
-      <c r="G854" t="inlineStr"/>
       <c r="H854" t="inlineStr">
         <is>
           <t>Oberoi Realty Fut 1839.80 45.80 BUY TGT 1930 SL 1840</t>
@@ -37179,7 +37113,6 @@
       <c r="F855" t="n">
         <v>422</v>
       </c>
-      <c r="G855" t="inlineStr"/>
       <c r="H855" t="inlineStr">
         <is>
           <t>विश्वेश चौहान की राय Kotak Bank Fut खरीदें PRICE 426.60 TARGET 432/436 STOP LOSS 422</t>
@@ -37221,7 +37154,6 @@
       <c r="F856" t="n">
         <v>422</v>
       </c>
-      <c r="G856" t="inlineStr"/>
       <c r="H856" t="inlineStr">
         <is>
           <t>विश्वेश चौहान की राय Kotak Bank Fut खरीदें PRICE 426.60 TARGET 432/436 STOP LOSS 422</t>
@@ -37254,11 +37186,9 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D857" t="inlineStr"/>
       <c r="E857" t="n">
         <v>5125</v>
       </c>
-      <c r="G857" t="inlineStr"/>
       <c r="H857" t="inlineStr">
         <is>
           <t>अनिल सिंघवी की सलाह
@@ -37296,14 +37226,12 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D858" t="inlineStr"/>
       <c r="E858" t="n">
         <v>5000</v>
       </c>
       <c r="F858" t="n">
         <v>5125</v>
       </c>
-      <c r="G858" t="inlineStr"/>
       <c r="H858" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -37341,14 +37269,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D859" t="inlineStr"/>
       <c r="E859" t="n">
         <v>12358</v>
       </c>
       <c r="F859" t="n">
         <v>12238</v>
       </c>
-      <c r="G859" t="inlineStr"/>
       <c r="H859" t="inlineStr">
         <is>
           <t>Bajaj Auto Fut 12163.00 BUY T 12238 S 12358 TARGET HIT</t>
@@ -37387,7 +37313,6 @@
       <c r="E860" t="n">
         <v>930</v>
       </c>
-      <c r="G860" t="inlineStr"/>
       <c r="H860" t="inlineStr">
         <is>
           <t>ANTELOPUS SELAN ENRGY LTD खरीदें PRICE 832.40 TARGET 930/950 STOP LOSS --</t>
@@ -37426,7 +37351,6 @@
       <c r="E861" t="n">
         <v>950</v>
       </c>
-      <c r="G861" t="inlineStr"/>
       <c r="H861" t="inlineStr">
         <is>
           <t>ANTELOPUS SELAN ENRGY LTD खरीदें PRICE 832.40 TARGET 930/950 STOP LOSS --</t>
@@ -37465,7 +37389,6 @@
       <c r="E862" t="n">
         <v>930</v>
       </c>
-      <c r="G862" t="inlineStr"/>
       <c r="H862" t="inlineStr">
         <is>
           <t>संदीप जैन की राय
@@ -37507,7 +37430,6 @@
       <c r="E863" t="n">
         <v>950</v>
       </c>
-      <c r="G863" t="inlineStr"/>
       <c r="H863" t="inlineStr">
         <is>
           <t>संदीप जैन की राय
@@ -37543,11 +37465,9 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D864" t="inlineStr"/>
       <c r="E864" t="n">
         <v>5000</v>
       </c>
-      <c r="G864" t="inlineStr"/>
       <c r="H864" t="inlineStr">
         <is>
           <t>OF THE DAY InterGlobe Aviation Fut 4947 SELL TGT 5000 TARGET HIT</t>
@@ -37586,7 +37506,6 @@
       <c r="E865" t="n">
         <v>3125</v>
       </c>
-      <c r="G865" t="inlineStr"/>
       <c r="H865" t="inlineStr">
         <is>
           <t>Interglobe Aviation Fut 4947.40 -99.00 SELL TARGET HIT 3125</t>
@@ -37619,14 +37538,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D866" t="inlineStr"/>
       <c r="E866" t="n">
         <v>371</v>
       </c>
       <c r="F866" t="n">
         <v>335</v>
       </c>
-      <c r="G866" t="inlineStr"/>
       <c r="H866" t="inlineStr">
         <is>
           <t>EMS Ltd 406.8 BUY TGT 371 SL 335 TARGET HIT</t>
@@ -37665,7 +37582,6 @@
       <c r="E867" t="n">
         <v>565</v>
       </c>
-      <c r="G867" t="inlineStr"/>
       <c r="H867" t="inlineStr">
         <is>
           <t>PICK OF THE DAY EMS Ltd 406.00 34.05 BUY TARGET HIT 565</t>
@@ -37698,14 +37614,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D868" t="inlineStr"/>
       <c r="E868" t="n">
         <v>3500</v>
       </c>
       <c r="F868" t="n">
         <v>3300</v>
       </c>
-      <c r="G868" t="inlineStr"/>
       <c r="H868" t="inlineStr">
         <is>
           <t>Centum Elec 3505 BUY TGT 3500 SL 3300 TARGET HIT</t>
@@ -37738,11 +37652,9 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D869" t="inlineStr"/>
       <c r="E869" t="n">
         <v>5600</v>
       </c>
-      <c r="G869" t="inlineStr"/>
       <c r="H869" t="inlineStr">
         <is>
           <t>अनिल सिंघवी की सलाह Hero Motocorp Fut 5408.50 -2.61% SELL TARGET HIT 5600</t>
@@ -37775,14 +37687,12 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D870" t="inlineStr"/>
       <c r="E870" t="n">
         <v>5000</v>
       </c>
       <c r="F870" t="n">
         <v>5125</v>
       </c>
-      <c r="G870" t="inlineStr"/>
       <c r="H870" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -37826,7 +37736,6 @@
       <c r="E871" t="n">
         <v>565</v>
       </c>
-      <c r="G871" t="inlineStr"/>
       <c r="H871" t="inlineStr">
         <is>
           <t>PICK OF THE DAY EMS Ltd 407.55 35.60 BUY TARGET HIT 565</t>
@@ -37859,14 +37768,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D872" t="inlineStr"/>
       <c r="E872" t="n">
         <v>371</v>
       </c>
       <c r="F872" t="n">
         <v>365</v>
       </c>
-      <c r="G872" t="inlineStr"/>
       <c r="H872" t="inlineStr">
         <is>
           <t>PICK OF THE DAY EMS Ltd 407.55 35.60 BUY TGT 371 SL 365</t>
@@ -37899,11 +37806,9 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D873" t="inlineStr"/>
       <c r="E873" t="n">
         <v>12550</v>
       </c>
-      <c r="G873" t="inlineStr"/>
       <c r="H873" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY Bajaj Auto Fut 12235.00 -1.17% SELL TARGET HIT 12550</t>
@@ -37936,14 +37841,12 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D874" t="inlineStr"/>
       <c r="E874" t="n">
         <v>12250</v>
       </c>
       <c r="F874" t="n">
         <v>12550</v>
       </c>
-      <c r="G874" t="inlineStr"/>
       <c r="H874" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -37981,11 +37884,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D875" t="inlineStr"/>
       <c r="E875" t="n">
         <v>3360</v>
       </c>
-      <c r="G875" t="inlineStr"/>
       <c r="H875" t="inlineStr">
         <is>
           <t>आस्था जैन
@@ -38023,7 +37924,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D876" t="inlineStr"/>
       <c r="E876" t="n">
         <v>3500</v>
       </c>
@@ -38072,14 +37972,12 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D877" t="inlineStr"/>
       <c r="E877" t="n">
         <v>5520</v>
       </c>
       <c r="F877" t="n">
         <v>5600</v>
       </c>
-      <c r="G877" t="inlineStr"/>
       <c r="H877" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -38117,11 +38015,9 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D878" t="inlineStr"/>
       <c r="E878" t="n">
         <v>5125</v>
       </c>
-      <c r="G878" t="inlineStr"/>
       <c r="H878" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -38165,7 +38061,6 @@
       <c r="E879" t="n">
         <v>3125</v>
       </c>
-      <c r="G879" t="inlineStr"/>
       <c r="H879" t="inlineStr">
         <is>
           <t>अनिल सिंघवी की सलाह
@@ -38203,14 +38098,12 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D880" t="inlineStr"/>
       <c r="E880" t="n">
         <v>5000</v>
       </c>
       <c r="F880" t="n">
         <v>5125</v>
       </c>
-      <c r="G880" t="inlineStr"/>
       <c r="H880" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -38248,14 +38141,12 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D881" t="inlineStr"/>
       <c r="E881" t="n">
         <v>5000</v>
       </c>
       <c r="F881" t="n">
         <v>5125</v>
       </c>
-      <c r="G881" t="inlineStr"/>
       <c r="H881" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -38299,7 +38190,6 @@
       <c r="E882" t="n">
         <v>565</v>
       </c>
-      <c r="G882" t="inlineStr"/>
       <c r="H882" t="inlineStr">
         <is>
           <t>अरुण शर्मा जैन
@@ -38337,7 +38227,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D883" t="inlineStr"/>
       <c r="E883" t="n">
         <v>365</v>
       </c>
@@ -38383,11 +38272,9 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D884" t="inlineStr"/>
       <c r="E884" t="n">
         <v>5600</v>
       </c>
-      <c r="G884" t="inlineStr"/>
       <c r="H884" t="inlineStr">
         <is>
           <t>अनिल सिंघवी की सलाह Hero Motocorp Fut 5428.00 -125.50 SELL TARGET HIT 5600</t>
@@ -38426,7 +38313,6 @@
       <c r="E885" t="n">
         <v>3600</v>
       </c>
-      <c r="G885" t="inlineStr"/>
       <c r="H885" t="inlineStr">
         <is>
           <t>अनिल सिंघवी की सलाह Hero Motocorp Fut 5428.00 -2.26% SELL TARGET HIT 3600</t>
@@ -38459,14 +38345,12 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="D886" t="inlineStr"/>
       <c r="E886" t="n">
         <v>5520</v>
       </c>
       <c r="F886" t="n">
         <v>5600</v>
       </c>
-      <c r="G886" t="inlineStr"/>
       <c r="H886" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -38510,7 +38394,6 @@
       <c r="E887" t="n">
         <v>9400</v>
       </c>
-      <c r="G887" t="inlineStr"/>
       <c r="H887" t="inlineStr">
         <is>
           <t>BROKERAGE CALLS
@@ -38553,7 +38436,6 @@
       <c r="E888" t="n">
         <v>9400</v>
       </c>
-      <c r="G888" t="inlineStr"/>
       <c r="H888" t="inlineStr">
         <is>
           <t>SBI Life 1728.30 11.00 0.63% Vol: 639 PRE-OPEN BROKERAGE CALLS BUY लक्ष्य ₹9400</t>
@@ -38592,7 +38474,6 @@
       <c r="E889" t="n">
         <v>2235</v>
       </c>
-      <c r="G889" t="inlineStr"/>
       <c r="H889" t="inlineStr">
         <is>
           <t>BROKERAGE CALLS BUY लक्ष्य ₹2235</t>
@@ -38631,7 +38512,6 @@
       <c r="E890" t="n">
         <v>440</v>
       </c>
-      <c r="G890" t="inlineStr"/>
       <c r="H890" t="inlineStr">
         <is>
           <t>Coal India 406.00 +4.40 HOLD लक्ष्य ₹440</t>
@@ -38670,7 +38550,6 @@
       <c r="E891" t="n">
         <v>440</v>
       </c>
-      <c r="G891" t="inlineStr"/>
       <c r="H891" t="inlineStr">
         <is>
           <t>Samvardhana Motherson 164.00 1.60 0.97% Vol: 19.98 k PRE-OPEN BROKERAGE CALLS HOLD लक्ष्य ₹440</t>
@@ -38712,7 +38591,6 @@
       <c r="F892" t="n">
         <v>12650</v>
       </c>
-      <c r="G892" t="inlineStr"/>
       <c r="H892" t="inlineStr">
         <is>
           <t>STOCK FTH D Bajaj Auto Futures SELL PRICE 12380 TARGET 2250, 12150, 1200 STOP LOSS 12650</t>
@@ -38754,7 +38632,6 @@
       <c r="F893" t="n">
         <v>12650</v>
       </c>
-      <c r="G893" t="inlineStr"/>
       <c r="H893" t="inlineStr">
         <is>
           <t>STOCK FTH D Bajaj Auto Futures SELL PRICE 12380 TARGET 2250, 12150, 1200 STOP LOSS 12650</t>
@@ -38796,7 +38673,6 @@
       <c r="F894" t="n">
         <v>12650</v>
       </c>
-      <c r="G894" t="inlineStr"/>
       <c r="H894" t="inlineStr">
         <is>
           <t>STOCK FTH D Bajaj Auto Futures SELL PRICE 12380 TARGET 2250, 12150, 1200 STOP LOSS 12650</t>
@@ -38838,7 +38714,6 @@
       <c r="F895" t="n">
         <v>271</v>
       </c>
-      <c r="G895" t="inlineStr"/>
       <c r="H895" t="inlineStr">
         <is>
           <t>MY CHOICE NLC INDIA B 281 271</t>
@@ -38877,7 +38752,6 @@
       <c r="E896" t="n">
         <v>510</v>
       </c>
-      <c r="G896" t="inlineStr"/>
       <c r="H896" t="inlineStr">
         <is>
           <t>MY CHOICE ICICI PRU LIFE B 510</t>
@@ -38916,7 +38790,6 @@
       <c r="E897" t="n">
         <v>867</v>
       </c>
-      <c r="G897" t="inlineStr"/>
       <c r="H897" t="inlineStr">
         <is>
           <t>MY CHOICE TITAGARH B 867</t>
@@ -38958,7 +38831,6 @@
       <c r="F898" t="n">
         <v>368</v>
       </c>
-      <c r="G898" t="inlineStr"/>
       <c r="H898" t="inlineStr">
         <is>
           <t>MY CHOICE HPCL FUT S 350 368</t>
@@ -39000,7 +38872,6 @@
       <c r="F899" t="n">
         <v>1240</v>
       </c>
-      <c r="G899" t="inlineStr"/>
       <c r="H899" t="inlineStr">
         <is>
           <t>PICK OF THE DAY UNO Minda Ltd BUY PRICE 1274.40 TARGET 1320/1340 STOP LOSS 1240</t>
@@ -39042,7 +38913,6 @@
       <c r="F900" t="n">
         <v>13500</v>
       </c>
-      <c r="G900" t="inlineStr"/>
       <c r="H900" t="inlineStr">
         <is>
           <t>विश्वेश चौहान की राय
@@ -39089,7 +38959,6 @@
       <c r="F901" t="n">
         <v>231</v>
       </c>
-      <c r="G901" t="inlineStr"/>
       <c r="H901" t="inlineStr">
         <is>
           <t>PICK OF THE DAY ONGC BUY PRICE 236.45 TARGET 240 STOP LOSS 231</t>
@@ -39131,7 +39000,6 @@
       <c r="F902" t="n">
         <v>3360</v>
       </c>
-      <c r="G902" t="inlineStr"/>
       <c r="H902" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Centum Elec BUY PRICE 3422.65 TARGET 3500 STOP LOSS 3360</t>
@@ -39173,7 +39041,6 @@
       <c r="F903" t="n">
         <v>12550</v>
       </c>
-      <c r="G903" t="inlineStr"/>
       <c r="H903" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY Bajaj Auto Futures SELL PRICE 12380 TARGET 12250, 12150, 12000 STOP LOSS 12550</t>
@@ -39215,7 +39082,6 @@
       <c r="F904" t="n">
         <v>12550</v>
       </c>
-      <c r="G904" t="inlineStr"/>
       <c r="H904" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY Bajaj Auto Futures SELL PRICE 12380 TARGET 12250, 12150, 12000 STOP LOSS 12550</t>
@@ -39257,7 +39123,6 @@
       <c r="F905" t="n">
         <v>12550</v>
       </c>
-      <c r="G905" t="inlineStr"/>
       <c r="H905" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY Bajaj Auto Futures SELL PRICE 12380 TARGET 12250, 12150, 12000 STOP LOSS 12550</t>
@@ -39299,7 +39164,6 @@
       <c r="F906" t="n">
         <v>5600</v>
       </c>
-      <c r="G906" t="inlineStr"/>
       <c r="H906" t="inlineStr">
         <is>
           <t>अनिल सिंघवी की सलाह
@@ -39343,7 +39207,6 @@
       <c r="E907" t="n">
         <v>9400</v>
       </c>
-      <c r="G907" t="inlineStr"/>
       <c r="H907" t="inlineStr">
         <is>
           <t>BROKERAGE CALLS
@@ -39386,7 +39249,6 @@
       <c r="E908" t="n">
         <v>183</v>
       </c>
-      <c r="G908" t="inlineStr"/>
       <c r="H908" t="inlineStr">
         <is>
           <t>BROKERAGE CALLS Lemon Tree Hotels 106.15 ACCUMULATE लक्ष्य ₹175 से बढ़ाकर ₹183</t>
@@ -39428,7 +39290,6 @@
       <c r="F909" t="n">
         <v>1424</v>
       </c>
-      <c r="G909" t="inlineStr"/>
       <c r="H909" t="inlineStr">
         <is>
           <t>INVESTMENT CONCORD BIO B 1610 1424</t>
@@ -39470,7 +39331,6 @@
       <c r="F910" t="n">
         <v>817</v>
       </c>
-      <c r="G910" t="inlineStr"/>
       <c r="H910" t="inlineStr">
         <is>
           <t>MY CHOICE TITAGARH B 867 817</t>
@@ -39512,7 +39372,6 @@
       <c r="F911" t="n">
         <v>488</v>
       </c>
-      <c r="G911" t="inlineStr"/>
       <c r="H911" t="inlineStr">
         <is>
           <t>MY CHOICE ICICI PRU LIFE B 510 488</t>
@@ -39554,7 +39413,6 @@
       <c r="F912" t="n">
         <v>248</v>
       </c>
-      <c r="G912" t="inlineStr"/>
       <c r="H912" t="inlineStr">
         <is>
           <t>CASH APTUS VALUE B 262 248</t>
@@ -39596,7 +39454,6 @@
       <c r="F913" t="n">
         <v>831</v>
       </c>
-      <c r="G913" t="inlineStr"/>
       <c r="H913" t="inlineStr">
         <is>
           <t>FUTURE MARICO FUT B 852 831</t>
@@ -39638,7 +39495,6 @@
       <c r="F914" t="n">
         <v>83</v>
       </c>
-      <c r="G914" t="inlineStr"/>
       <c r="H914" t="inlineStr">
         <is>
           <t>FUNDA NMDC B 92 83</t>
@@ -39677,7 +39533,6 @@
       <c r="E915" t="n">
         <v>520</v>
       </c>
-      <c r="G915" t="inlineStr"/>
       <c r="H915" t="inlineStr">
         <is>
           <t>INVESTMENT TATA MOTORS CV B 520 12 MONTH</t>
@@ -39719,7 +39574,6 @@
       <c r="F916" t="n">
         <v>170</v>
       </c>
-      <c r="G916" t="inlineStr"/>
       <c r="H916" t="inlineStr">
         <is>
           <t>NEWS IMPACT SRI LOTUS DEVELOPERS B 186 170</t>
@@ -39761,7 +39615,6 @@
       <c r="F917" t="n">
         <v>322</v>
       </c>
-      <c r="G917" t="inlineStr"/>
       <c r="H917" t="inlineStr">
         <is>
           <t>MY CHOICE BPCL FUT S 310 322</t>
@@ -39800,7 +39653,6 @@
       <c r="E918" t="n">
         <v>1086</v>
       </c>
-      <c r="G918" t="inlineStr"/>
       <c r="H918" t="inlineStr">
         <is>
           <t>NEWS IMPACT SRI LOTUS DEVELOPERS B 1086 170</t>
@@ -39839,7 +39691,6 @@
       <c r="F919" t="n">
         <v>3350</v>
       </c>
-      <c r="G919" t="inlineStr"/>
       <c r="H919" t="inlineStr">
         <is>
           <t>MY CHOICE HDFC BANK S 3350</t>
@@ -39881,7 +39732,6 @@
       <c r="F920" t="n">
         <v>5610</v>
       </c>
-      <c r="G920" t="inlineStr"/>
       <c r="H920" t="inlineStr">
         <is>
           <t>FUTURE HERO MOTO FUT S 5446 5610</t>
@@ -39920,7 +39770,6 @@
       <c r="E921" t="n">
         <v>12800</v>
       </c>
-      <c r="G921" t="inlineStr"/>
       <c r="H921" t="inlineStr">
         <is>
           <t>FUNDA BAJAJ AUTO B 12800 3 MONTH</t>
@@ -39962,7 +39811,6 @@
       <c r="F922" t="n">
         <v>271</v>
       </c>
-      <c r="G922" t="inlineStr"/>
       <c r="H922" t="inlineStr">
         <is>
           <t>MY CHOICE
@@ -40009,7 +39857,6 @@
       <c r="F923" t="n">
         <v>488</v>
       </c>
-      <c r="G923" t="inlineStr"/>
       <c r="H923" t="inlineStr">
         <is>
           <t>ICICI Pru खरीदें PRICE 495.45 TARGET 510 STOP LOSS 488</t>
@@ -40051,7 +39898,6 @@
       <c r="F924" t="n">
         <v>817</v>
       </c>
-      <c r="G924" t="inlineStr"/>
       <c r="H924" t="inlineStr">
         <is>
           <t>अंश के शेयर Titagarh Rail खरीदें PRICE 833.95 TARGET 867 STOP LOSS 817</t>
@@ -40093,7 +39939,6 @@
       <c r="F925" t="n">
         <v>322</v>
       </c>
-      <c r="G925" t="inlineStr"/>
       <c r="H925" t="inlineStr">
         <is>
           <t>MY CHOICE
@@ -40137,7 +39982,6 @@
       <c r="E926" t="n">
         <v>310</v>
       </c>
-      <c r="G926" t="inlineStr"/>
       <c r="H926" t="inlineStr">
         <is>
           <t>MY CHOICE
@@ -40182,7 +40026,6 @@
       <c r="F927" t="n">
         <v>368</v>
       </c>
-      <c r="G927" t="inlineStr"/>
       <c r="H927" t="inlineStr">
         <is>
           <t>MY CHOICE HPCL Fut बेचें PRICE 362.85 TARGET 350 STOP LOSS 368</t>
@@ -40224,7 +40067,6 @@
       <c r="F928" t="n">
         <v>170</v>
       </c>
-      <c r="G928" t="inlineStr"/>
       <c r="H928" t="inlineStr">
         <is>
           <t>खबर के दम पर
@@ -40268,7 +40110,6 @@
       <c r="E929" t="n">
         <v>186</v>
       </c>
-      <c r="G929" t="inlineStr"/>
       <c r="H929" t="inlineStr">
         <is>
           <t>खबर के दम पर
@@ -40313,7 +40154,6 @@
       <c r="F930" t="n">
         <v>83</v>
       </c>
-      <c r="G930" t="inlineStr"/>
       <c r="H930" t="inlineStr">
         <is>
           <t>FUNDA PICK NMDC खरीदें PRICE 85.69 TARGET 92 STOP LOSS 83</t>
@@ -40352,7 +40192,6 @@
       <c r="E931" t="n">
         <v>12800</v>
       </c>
-      <c r="G931" t="inlineStr"/>
       <c r="H931" t="inlineStr">
         <is>
           <t>FUNDA PICK
@@ -40399,7 +40238,6 @@
       <c r="F932" t="n">
         <v>5610</v>
       </c>
-      <c r="G932" t="inlineStr"/>
       <c r="H932" t="inlineStr">
         <is>
           <t>आज का FUTURE
@@ -40446,7 +40284,6 @@
       <c r="F933" t="n">
         <v>831</v>
       </c>
-      <c r="G933" t="inlineStr"/>
       <c r="H933" t="inlineStr">
         <is>
           <t>आज का FUTURE
@@ -40493,7 +40330,6 @@
       <c r="F934" t="n">
         <v>248</v>
       </c>
-      <c r="G934" t="inlineStr"/>
       <c r="H934" t="inlineStr">
         <is>
           <t>CASH का शेयर Aptus Value खरीदें PRICE 253.36 TARGET 262 STOP LOSS 248</t>
@@ -40535,7 +40371,6 @@
       <c r="F935" t="n">
         <v>2846</v>
       </c>
-      <c r="G935" t="inlineStr"/>
       <c r="H935" t="inlineStr">
         <is>
           <t>CASH का शेयर
@@ -40582,7 +40417,6 @@
       <c r="F936" t="n">
         <v>322</v>
       </c>
-      <c r="G936" t="inlineStr"/>
       <c r="H936" t="inlineStr">
         <is>
           <t>सिद्धार्थ राय मंगला की राय Eternal (Zomato) खरीदें PRICE 327.75 TARGET 340/350 STOP LOSS 322</t>
@@ -40621,7 +40455,6 @@
       <c r="E937" t="n">
         <v>4650</v>
       </c>
-      <c r="G937" t="inlineStr"/>
       <c r="H937" t="inlineStr">
         <is>
           <t>सिटी
@@ -40664,7 +40497,6 @@
       <c r="E938" t="n">
         <v>2120</v>
       </c>
-      <c r="G938" t="inlineStr"/>
       <c r="H938" t="inlineStr">
         <is>
           <t>Sun Pharma 1929 BUY लक्ष्य ₹2120</t>
@@ -40681,8 +40513,2733 @@
         </is>
       </c>
     </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:42:42</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>INDIANB</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr"/>
+      <c r="E939" t="n">
+        <v>910</v>
+      </c>
+      <c r="F939" t="n">
+        <v>879</v>
+      </c>
+      <c r="G939" t="inlineStr"/>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>शुभ 'मंगला' शेयर
+Indian Bank
+खरीदें
+PRICE 893.80
+TARGET 910/925
+STOP LOSS 879</t>
+        </is>
+      </c>
+      <c r="I939" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J939" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:42:40</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>INDIANB</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr"/>
+      <c r="E940" t="n">
+        <v>925</v>
+      </c>
+      <c r="F940" t="n">
+        <v>879</v>
+      </c>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>Siddharth Ray Mangla</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>सिद्धार्थ राय मंगला की राय
+Indian Bank
+खरीदें
+PRICE ▶ 893.85
+TARGET ▶ 910/925
+STOP LOSS ▶ 879</t>
+        </is>
+      </c>
+      <c r="I940" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J940" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:37:57</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>INDIANHUME</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr"/>
+      <c r="E941" t="n">
+        <v>360</v>
+      </c>
+      <c r="G941" t="inlineStr"/>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>Indian Hume Pipe 395.00 1.62% BUY TARGET HIT 360</t>
+        </is>
+      </c>
+      <c r="I941" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J941" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:37:53</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>INDIANHUME</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr"/>
+      <c r="E942" t="n">
+        <v>405</v>
+      </c>
+      <c r="F942" t="n">
+        <v>360</v>
+      </c>
+      <c r="G942" t="inlineStr"/>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>Indian Hume Pipe ▲ 396.85 8.15 BUY TGT 405 SL 360</t>
+        </is>
+      </c>
+      <c r="I942" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J942" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:36:25</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>NGLFINE</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr"/>
+      <c r="E943" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G943" t="inlineStr"/>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>संदीप जैन की राय
+NGL Fine Chem Ltd
+खरीदें
+PRICE → 2836.00
+TARGET → 3190
+STOP LOSS → ---</t>
+        </is>
+      </c>
+      <c r="I943" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J943" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:36:24</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>NGLFINE</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr"/>
+      <c r="E944" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G944" t="inlineStr"/>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>संदीप जैन की राय
+NGL Fine Chem Ltd
+खरीदें
+PRICE ▶ 2835.10
+TARGET ▶ 3190
+STOP LOSS ▶ ---</t>
+        </is>
+      </c>
+      <c r="I944" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J944" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:32:00</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>INDIANHUME</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D945" t="n">
+        <v>398</v>
+      </c>
+      <c r="E945" t="n">
+        <v>405</v>
+      </c>
+      <c r="G945" t="inlineStr"/>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>Indian Hume Pipe 401.15 BUY TGT 405 TARGET HIT</t>
+        </is>
+      </c>
+      <c r="I945" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J945" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:32:00</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>INDIANHUME</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D946" t="n">
+        <v>398</v>
+      </c>
+      <c r="E946" t="n">
+        <v>405</v>
+      </c>
+      <c r="F946" t="n">
+        <v>360</v>
+      </c>
+      <c r="G946" t="inlineStr"/>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>Indian Hume Pipe 401.15 12.45 BUY TGT 405 SL 360</t>
+        </is>
+      </c>
+      <c r="I946" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J946" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:28:47</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr"/>
+      <c r="E947" t="n">
+        <v>189.04</v>
+      </c>
+      <c r="G947" t="inlineStr"/>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>Union Bank 189.04 INVESTMENT PICK 106.00 28/01/2025 RECO PRICE RETURN TILL NOW 83.04 78.34%</t>
+        </is>
+      </c>
+      <c r="I947" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J947" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:28:00</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>INDIANHUME</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D948" t="n">
+        <v>401.5</v>
+      </c>
+      <c r="E948" t="n">
+        <v>560</v>
+      </c>
+      <c r="G948" t="inlineStr"/>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>Indian Hume Pipe 400.00 11.30 BUY TARGET HIT 560</t>
+        </is>
+      </c>
+      <c r="I948" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J948" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:28:00</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>INDIANHUME</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D949" t="n">
+        <v>401.5</v>
+      </c>
+      <c r="E949" t="n">
+        <v>405</v>
+      </c>
+      <c r="F949" t="n">
+        <v>360</v>
+      </c>
+      <c r="G949" t="inlineStr">
+        <is>
+          <t>Vikas Sethi</t>
+        </is>
+      </c>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>सदाबहार सेठी सा'ब
+Indian Hume Pipe
+400.00 11.30
+BUY
+TGT 405
+SL 360</t>
+        </is>
+      </c>
+      <c r="I949" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J949" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:27:00</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D950" t="n">
+        <v>537.5</v>
+      </c>
+      <c r="E950" t="n">
+        <v>545</v>
+      </c>
+      <c r="F950" t="n">
+        <v>530</v>
+      </c>
+      <c r="G950" t="inlineStr"/>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>सुमित बगडिया की राय HDFC Life खरीदें PRICE 537.10 TARGET 545/555 STOP LOSS 530</t>
+        </is>
+      </c>
+      <c r="I950" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J950" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:27:00</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D951" t="n">
+        <v>537.5</v>
+      </c>
+      <c r="E951" t="n">
+        <v>555</v>
+      </c>
+      <c r="F951" t="n">
+        <v>530</v>
+      </c>
+      <c r="G951" t="inlineStr"/>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>सुमित बगडिया की राय HDFC Life खरीदें PRICE 537.10 TARGET 545/555 STOP LOSS 530</t>
+        </is>
+      </c>
+      <c r="I951" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J951" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:26:00</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D952" t="n">
+        <v>2970.3</v>
+      </c>
+      <c r="E952" t="n">
+        <v>3010</v>
+      </c>
+      <c r="F952" t="n">
+        <v>2945</v>
+      </c>
+      <c r="G952" t="inlineStr"/>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>शुभ 'मंगला' शेयर Muthoot Finance खरीदें PRICE 2969.00 TARGET 3010/3030 STOP LOSS 2945</t>
+        </is>
+      </c>
+      <c r="I952" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J952" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:26:00</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D953" t="n">
+        <v>2970.3</v>
+      </c>
+      <c r="E953" t="n">
+        <v>3030</v>
+      </c>
+      <c r="F953" t="n">
+        <v>2945</v>
+      </c>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>Siddharth Ray Mangla</t>
+        </is>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>सिद्धार्थ राय मंगला की राय Muthoot Finance खरीदें PRICE 2969.90 TARGET 3010/3030 STOP LOSS 2945</t>
+        </is>
+      </c>
+      <c r="I953" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J953" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:26:00</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D954" t="n">
+        <v>2970.3</v>
+      </c>
+      <c r="E954" t="n">
+        <v>3010</v>
+      </c>
+      <c r="F954" t="n">
+        <v>2945</v>
+      </c>
+      <c r="G954" t="inlineStr"/>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>शुभ 'मंगला' शरीर Muthoot Finance खरीदें PRICE 2968.40 TARGET 3010/3030 STOP LOSS 2945</t>
+        </is>
+      </c>
+      <c r="I954" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J954" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:26:00</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D955" t="n">
+        <v>2970.3</v>
+      </c>
+      <c r="E955" t="n">
+        <v>3030</v>
+      </c>
+      <c r="F955" t="n">
+        <v>2945</v>
+      </c>
+      <c r="G955" t="inlineStr"/>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>शुभ 'मंगला' शरीर Muthoot Finance खरीदें PRICE 2968.40 TARGET 3010/3030 STOP LOSS 2945</t>
+        </is>
+      </c>
+      <c r="I955" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J955" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:23:51</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>BANKBARODA29SEP26</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr"/>
+      <c r="E956" t="n">
+        <v>90</v>
+      </c>
+      <c r="F956" t="n">
+        <v>81</v>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>Somil Mehta</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>सोमिल मेहता की राय
+Bank of Maha Fut
+खरीदें
+PRICE ▶ 85.37
+TARGET ▶ 90
+STOP LOSS ▶ 81</t>
+        </is>
+      </c>
+      <c r="I956" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J956" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:23:00</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D957" t="n">
+        <v>1032.6</v>
+      </c>
+      <c r="E957" t="n">
+        <v>1070</v>
+      </c>
+      <c r="F957" t="n">
+        <v>1015</v>
+      </c>
+      <c r="G957" t="inlineStr"/>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>सुमित बगडिया की राय
+SBI
+खरीदें
+PRICE → 1030.30
+TARGET → 1050/1070
+STOP LOSS → 1015</t>
+        </is>
+      </c>
+      <c r="I957" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J957" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:23:00</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D958" t="n">
+        <v>1032.6</v>
+      </c>
+      <c r="E958" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F958" t="n">
+        <v>1015</v>
+      </c>
+      <c r="G958" t="inlineStr"/>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>सुमित बगडिया की राय
+SBI
+खरीदें
+PRICE → 1030.30
+TARGET → 1050/1070
+STOP LOSS → 1015</t>
+        </is>
+      </c>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J958" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:16:00</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>WELCORP</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D959" t="n">
+        <v>2575</v>
+      </c>
+      <c r="E959" t="n">
+        <v>3250</v>
+      </c>
+      <c r="G959" t="inlineStr"/>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>BROKERAGE CALLS
+Welspun Corp
+2554.70 +31.20
+BUY
+लक्ष्य ₹3250</t>
+        </is>
+      </c>
+      <c r="I959" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J959" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>RBLBANK29SEP26</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D960" t="n">
+        <v>399.85</v>
+      </c>
+      <c r="E960" t="n">
+        <v>405</v>
+      </c>
+      <c r="F960" t="n">
+        <v>385</v>
+      </c>
+      <c r="G960" t="inlineStr"/>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह RBL Bank Futures BUY PRICE 392 TARGET 396, 400, 405 STOP LOSS 385</t>
+        </is>
+      </c>
+      <c r="I960" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J960" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>RBLBANK29SEP26</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D961" t="n">
+        <v>399.85</v>
+      </c>
+      <c r="E961" t="n">
+        <v>400</v>
+      </c>
+      <c r="F961" t="n">
+        <v>385</v>
+      </c>
+      <c r="G961" t="inlineStr"/>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह RBL Bank Futures BUY PRICE 392 TARGET 396, 400, 405 STOP LOSS 385</t>
+        </is>
+      </c>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J961" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>FSL</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D962" t="n">
+        <v>270.15</v>
+      </c>
+      <c r="E962" t="n">
+        <v>279</v>
+      </c>
+      <c r="F962" t="n">
+        <v>266.5</v>
+      </c>
+      <c r="G962" t="inlineStr"/>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>MY CHOICE FIRSTSOURCE B 279 266.5</t>
+        </is>
+      </c>
+      <c r="I962" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J962" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D963" t="n">
+        <v>1438.3</v>
+      </c>
+      <c r="E963" t="n">
+        <v>1454</v>
+      </c>
+      <c r="F963" t="n">
+        <v>1411</v>
+      </c>
+      <c r="G963" t="inlineStr"/>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>MY CHOICE ICICI BANK B 1454 1411</t>
+        </is>
+      </c>
+      <c r="I963" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J963" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D964" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="E964" t="n">
+        <v>192</v>
+      </c>
+      <c r="F964" t="n">
+        <v>182</v>
+      </c>
+      <c r="G964" t="inlineStr"/>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY Union Bank BUY PRICE 186.86 TARGET 192/195 STOP LOSS 182</t>
+        </is>
+      </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J964" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D965" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="E965" t="n">
+        <v>195</v>
+      </c>
+      <c r="F965" t="n">
+        <v>182</v>
+      </c>
+      <c r="G965" t="inlineStr"/>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY Union Bank BUY PRICE 186.86 TARGET 192/195 STOP LOSS 182</t>
+        </is>
+      </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J965" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:16:00</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D966" t="n">
+        <v>208.6</v>
+      </c>
+      <c r="E966" t="n">
+        <v>212</v>
+      </c>
+      <c r="F966" t="n">
+        <v>204</v>
+      </c>
+      <c r="G966" t="inlineStr"/>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY Adani Power B PRICE 207.70 TARGET 212 STOP LOSS 204</t>
+        </is>
+      </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J966" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:17:00</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D967" t="n">
+        <v>268.6</v>
+      </c>
+      <c r="E967" t="n">
+        <v>272</v>
+      </c>
+      <c r="F967" t="n">
+        <v>265</v>
+      </c>
+      <c r="G967" t="inlineStr"/>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY Power Grid BUY PRICE 267.50 TARGET 272 STOP LOSS 265</t>
+        </is>
+      </c>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J967" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>ICICIPRULI</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D968" t="n">
+        <v>501.7</v>
+      </c>
+      <c r="E968" t="n">
+        <v>510</v>
+      </c>
+      <c r="F968" t="n">
+        <v>494</v>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>Vikas Sethi</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>विकास सेठी की राय ICICI Pru BUY PRICE 499.50 TARGET 510 STOP LOSS 494</t>
+        </is>
+      </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J968" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:16:00</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>FEDERALBNK29SEP26</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D969" t="n">
+        <v>356.9</v>
+      </c>
+      <c r="E969" t="n">
+        <v>375</v>
+      </c>
+      <c r="F969" t="n">
+        <v>346</v>
+      </c>
+      <c r="G969" t="inlineStr"/>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY
+Federal Bank Fut
+BUY
+PRICE ▶ 354.65
+TARGET ▶ 375
+STOP LOSS ▶ 346</t>
+        </is>
+      </c>
+      <c r="I969" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J969" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>JSWENERGY29SEP26</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D970" t="n">
+        <v>544.85</v>
+      </c>
+      <c r="E970" t="n">
+        <v>557</v>
+      </c>
+      <c r="F970" t="n">
+        <v>530</v>
+      </c>
+      <c r="G970" t="inlineStr"/>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह JSW Energy Futures BUY PRICE 541 TARGET 545, 550, 557 STOP LOSS 530</t>
+        </is>
+      </c>
+      <c r="I970" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J970" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>JSWENERGY29SEP26</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D971" t="n">
+        <v>544.85</v>
+      </c>
+      <c r="E971" t="n">
+        <v>550</v>
+      </c>
+      <c r="F971" t="n">
+        <v>530</v>
+      </c>
+      <c r="G971" t="inlineStr"/>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह JSW Energy Futures BUY PRICE 541 TARGET 545, 550, 557 STOP LOSS 530</t>
+        </is>
+      </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J971" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:16:00</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>FEDERALBNK29SEP26</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D972" t="n">
+        <v>356.9</v>
+      </c>
+      <c r="E972" t="n">
+        <v>365</v>
+      </c>
+      <c r="F972" t="n">
+        <v>347</v>
+      </c>
+      <c r="G972" t="inlineStr"/>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह
+Federal Bank Futures
+UY
+PRICE ▶ 354.5
+TARGET ▶ 358, 361, 365
+STOP LOSS ▶ 347</t>
+        </is>
+      </c>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J972" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:16:00</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>FEDERALBNK29SEP26</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D973" t="n">
+        <v>356.9</v>
+      </c>
+      <c r="E973" t="n">
+        <v>361</v>
+      </c>
+      <c r="F973" t="n">
+        <v>347</v>
+      </c>
+      <c r="G973" t="inlineStr"/>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह
+Federal Bank Futures
+UY
+PRICE ▶ 354.5
+TARGET ▶ 358, 361, 365
+STOP LOSS ▶ 347</t>
+        </is>
+      </c>
+      <c r="I973" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J973" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D974" t="n">
+        <v>269.3</v>
+      </c>
+      <c r="E974" t="n">
+        <v>273</v>
+      </c>
+      <c r="F974" t="n">
+        <v>264</v>
+      </c>
+      <c r="G974" t="inlineStr"/>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>NEWS IMPACT POWER GRID B 273 264</t>
+        </is>
+      </c>
+      <c r="I974" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J974" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>GODFRYPHLP</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D975" t="n">
+        <v>2041</v>
+      </c>
+      <c r="E975" t="n">
+        <v>2230</v>
+      </c>
+      <c r="F975" t="n">
+        <v>1926</v>
+      </c>
+      <c r="G975" t="inlineStr"/>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>INVESTMENT GODFREY PHILLIPS B 2230 1926</t>
+        </is>
+      </c>
+      <c r="I975" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J975" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>ZENSARTECH</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D976" t="n">
+        <v>463.9</v>
+      </c>
+      <c r="E976" t="n">
+        <v>474</v>
+      </c>
+      <c r="F976" t="n">
+        <v>455</v>
+      </c>
+      <c r="G976" t="inlineStr"/>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>MY CHOICE ZENSAR TECH B 474 455</t>
+        </is>
+      </c>
+      <c r="I976" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J976" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>UPL29SEP26</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D977" t="n">
+        <v>579.9</v>
+      </c>
+      <c r="E977" t="n">
+        <v>593</v>
+      </c>
+      <c r="F977" t="n">
+        <v>573</v>
+      </c>
+      <c r="G977" t="inlineStr"/>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>FUTURE UPL FUT B 593 573</t>
+        </is>
+      </c>
+      <c r="I977" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J977" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>PHOENIXLTD</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D978" t="n">
+        <v>1923</v>
+      </c>
+      <c r="E978" t="n">
+        <v>2060</v>
+      </c>
+      <c r="F978" t="n">
+        <v>1857</v>
+      </c>
+      <c r="G978" t="inlineStr"/>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>TECHNO PHOENIX MILLS B 2060 1857</t>
+        </is>
+      </c>
+      <c r="I978" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J978" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>KIRLOSENG</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D979" t="n">
+        <v>2173.8</v>
+      </c>
+      <c r="E979" t="n">
+        <v>2215</v>
+      </c>
+      <c r="F979" t="n">
+        <v>2150</v>
+      </c>
+      <c r="G979" t="inlineStr"/>
+      <c r="H979" t="inlineStr">
+        <is>
+          <t>MY CHOICE KIRLOSKAR OIL ENGINES B 2215 2150</t>
+        </is>
+      </c>
+      <c r="I979" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J979" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D980" t="n">
+        <v>422</v>
+      </c>
+      <c r="E980" t="n">
+        <v>460</v>
+      </c>
+      <c r="G980" t="inlineStr"/>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>INVESTMENT COAL INDIA B 460 12 MONTH</t>
+        </is>
+      </c>
+      <c r="I980" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J980" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D981" t="n">
+        <v>425</v>
+      </c>
+      <c r="E981" t="n">
+        <v>432</v>
+      </c>
+      <c r="F981" t="n">
+        <v>418</v>
+      </c>
+      <c r="G981" t="inlineStr"/>
+      <c r="H981" t="inlineStr">
+        <is>
+          <t>MY CHOICE KOTAK BANK B 432 418</t>
+        </is>
+      </c>
+      <c r="I981" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J981" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>FEDERALBNK29SEP26</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D982" t="n">
+        <v>356.7</v>
+      </c>
+      <c r="E982" t="n">
+        <v>361</v>
+      </c>
+      <c r="F982" t="n">
+        <v>349</v>
+      </c>
+      <c r="G982" t="inlineStr"/>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>FUTURE FEDERAL BANK FUT B 361 349</t>
+        </is>
+      </c>
+      <c r="I982" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J982" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>OLAELEC</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D983" t="n">
+        <v>39.35</v>
+      </c>
+      <c r="E983" t="n">
+        <v>41</v>
+      </c>
+      <c r="F983" t="n">
+        <v>37</v>
+      </c>
+      <c r="G983" t="inlineStr"/>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>CASH OLA ELECTRIC B 41 37</t>
+        </is>
+      </c>
+      <c r="I983" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J983" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>LLOYDSME</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D984" t="n">
+        <v>1818</v>
+      </c>
+      <c r="E984" t="n">
+        <v>1852</v>
+      </c>
+      <c r="F984" t="n">
+        <v>1794</v>
+      </c>
+      <c r="G984" t="inlineStr"/>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>MY CHOICE Lloyds Metals &amp; Energy Ltd खरीदें PRICE 1813.00 TARGET 1852 STOP LOSS 1794</t>
+        </is>
+      </c>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J984" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>FSL</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D985" t="n">
+        <v>270.15</v>
+      </c>
+      <c r="E985" t="n">
+        <v>279</v>
+      </c>
+      <c r="F985" t="n">
+        <v>266.5</v>
+      </c>
+      <c r="G985" t="inlineStr"/>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>अंश के शेयर Firstsource खरीदें PRICE 270.40 TARGET 279 STOP LOSS 266.5</t>
+        </is>
+      </c>
+      <c r="I985" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J985" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>KIRLOSENG</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D986" t="n">
+        <v>2173.8</v>
+      </c>
+      <c r="E986" t="n">
+        <v>2215</v>
+      </c>
+      <c r="F986" t="n">
+        <v>2150</v>
+      </c>
+      <c r="G986" t="inlineStr"/>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>पूजा के शेयर Kirloskar Oil खरीदें PRICE 2160.90 TARGET 2215 STOP LOSS 2150</t>
+        </is>
+      </c>
+      <c r="I986" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J986" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D987" t="n">
+        <v>1438.3</v>
+      </c>
+      <c r="E987" t="n">
+        <v>1454</v>
+      </c>
+      <c r="F987" t="n">
+        <v>1411</v>
+      </c>
+      <c r="G987" t="inlineStr"/>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>MY CHOICE ICICI Bank खरीदें PRICE 1426.50 TARGET 1454 STOP LOSS 1411</t>
+        </is>
+      </c>
+      <c r="I987" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J987" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D988" t="n">
+        <v>425</v>
+      </c>
+      <c r="E988" t="n">
+        <v>432</v>
+      </c>
+      <c r="F988" t="n">
+        <v>418</v>
+      </c>
+      <c r="G988" t="inlineStr"/>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>Kotak Bank खरीदें PRICE 423.50 TARGET 432 STOP LOSS 418</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J988" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:17:00</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D989" t="n">
+        <v>268.6</v>
+      </c>
+      <c r="E989" t="n">
+        <v>273</v>
+      </c>
+      <c r="F989" t="n">
+        <v>264</v>
+      </c>
+      <c r="G989" t="inlineStr"/>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>Power Grid खरीदें PRICE 266.80 TARGET 273 STOP LOSS 264</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J989" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D990" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="E990" t="n">
+        <v>460</v>
+      </c>
+      <c r="G990" t="inlineStr"/>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>इन्वेस्टमेंट PICK Coal India खरीदें PRICE 417.85 TARGET 460 DURATION 12 महीने</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J990" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>GODFRYPHLP</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D991" t="n">
+        <v>2041</v>
+      </c>
+      <c r="E991" t="n">
+        <v>2230</v>
+      </c>
+      <c r="F991" t="n">
+        <v>1926</v>
+      </c>
+      <c r="G991" t="inlineStr"/>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>इन्वेस्टमेंट PICK Godfrey Phillips खरीदें PRICE 2025.40 TARGET 2230 STOP LOSS 1926</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J991" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:16:00</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D992" t="n">
+        <v>366.1</v>
+      </c>
+      <c r="E992" t="n">
+        <v>371</v>
+      </c>
+      <c r="F992" t="n">
+        <v>360</v>
+      </c>
+      <c r="G992" t="inlineStr"/>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>पूजा के शेयर Tata Power खरीदें PRICE 364.00 TARGET 371 STOP LOSS 360</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J992" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>PHOENIXLTD</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D993" t="n">
+        <v>1923</v>
+      </c>
+      <c r="E993" t="n">
+        <v>2060</v>
+      </c>
+      <c r="F993" t="n">
+        <v>1857</v>
+      </c>
+      <c r="G993" t="inlineStr"/>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>TECHNO PICK Phoenix Mills खरीदें PRICE 1920.10 TARGET 2060 STOP LOSS 1857</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J993" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D994" t="n">
+        <v>2172</v>
+      </c>
+      <c r="E994" t="n">
+        <v>2438</v>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>अंश के शेयर मॉर्गन स्टैनली की ओवरवेट राय, लक्ष्य ₹2131 से बढ़ाकर ₹2438 Hyundai Motor 2154.40 1.17%</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J994" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>FEDERALBNK29SEP26</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D995" t="n">
+        <v>356.7</v>
+      </c>
+      <c r="E995" t="n">
+        <v>361</v>
+      </c>
+      <c r="F995" t="n">
+        <v>349</v>
+      </c>
+      <c r="G995" t="inlineStr"/>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>पूजा के शेयर
+Federal Bank Fut
+खरीदें
+PRICE 354.65
+TARGET 361
+STOP LOSS 349</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J995" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>ICICIPRULI</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D996" t="n">
+        <v>501.7</v>
+      </c>
+      <c r="E996" t="n">
+        <v>1470</v>
+      </c>
+      <c r="G996" t="inlineStr"/>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>STOCKS IN NEWS
+ICICI Bank 1426.50 -0.80%
+ICICI Pru का 2 % हिस्सा ₹ 1470 Cr में खरीदा</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J996" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D997" t="n">
+        <v>1864.9</v>
+      </c>
+      <c r="E997" t="n">
+        <v>1890</v>
+      </c>
+      <c r="F997" t="n">
+        <v>1835</v>
+      </c>
+      <c r="G997" t="inlineStr"/>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>TRADING CALL Laurus Labs खरीदें PRICE 1864.00 TARGET 1890/1910 STOP LOSS 1835</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J997" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D998" t="n">
+        <v>1864.9</v>
+      </c>
+      <c r="E998" t="n">
+        <v>1910</v>
+      </c>
+      <c r="F998" t="n">
+        <v>1835</v>
+      </c>
+      <c r="G998" t="inlineStr"/>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>TRADING CALL Laurus Labs खरीदें PRICE 1864.00 TARGET 1890/1910 STOP LOSS 1835</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J998" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D999" t="n">
+        <v>1681.8</v>
+      </c>
+      <c r="E999" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G999" t="inlineStr"/>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>BROKERAGE CALLS
+Adani Ports
+1672.70 +25.20
+OVERWEIGHT
+लक्ष्य ₹2000</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J999" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1000" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="E1000" t="n">
+        <v>465</v>
+      </c>
+      <c r="G1000" t="inlineStr"/>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>BROKERAGE CALL
+Coal India
+417.85 +4.05%
+BUY
+लक्ष्य ₹430 से बढ़ाकर ₹465</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1000" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>SHILPAMED</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1001" t="n">
+        <v>935</v>
+      </c>
+      <c r="E1001" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G1001" t="inlineStr"/>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>LUNG-TERM CALL Shilpa Medicare BUY TARGET 1200 DURATION 12 महीने Shilpa Medicare 928.55 4.37%</t>
+        </is>
+      </c>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1001" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-09-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>HAPPSTMNDS</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1002" t="n">
+        <v>356</v>
+      </c>
+      <c r="E1002" t="n">
+        <v>550</v>
+      </c>
+      <c r="G1002" t="inlineStr"/>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>सुदीप बंदोपाध्याय की पसंद Happiest Minds BUY TARGET 550 DURATION 12 महीने Happiest Minds 354.85 7.85</t>
+        </is>
+      </c>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1002" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J938"/>
+  <autoFilter ref="A1:J1002"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>